<commit_message>
replace J2 1734715-2 -> 5569262-1 due to parts availability
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_A_MAX11331_Daugther/Rev03/BOM_JLC/BOM_JLC_UZ_A_MAX11331_Daugther_SMD_Assembly_Rev03.xlsx
+++ b/Project Outputs for UZ_A_MAX11331_Daugther/Rev03/BOM_JLC/BOM_JLC_UZ_A_MAX11331_Daugther_SMD_Assembly_Rev03.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ga92wum\git\UltraZohm\PCB\UZ_A_MAX11331_Main\Project Outputs for UZ_A_MAX11331_Daugther\Rev03\BOM_JLC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ga92wum\git\UltraZohm\PCB\UZ_A_MAX11331_Daugther\Project Outputs for UZ_A_MAX11331_Daugther\Rev03\BOM_JLC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A38B059-0A41-428C-AF1F-0E425F3A61BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8DE81117-AABD-45F0-B5BA-491B34918D94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{FE9CF728-2853-4E42-AD22-A280F78FC907}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{E28598CA-BEFF-49BF-B6AA-06D89354CDA5}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC_UZ_A_MAX11331_Daugther_" sheetId="1" r:id="rId1"/>
@@ -164,7 +164,7 @@
     <t>RJ45 - 4x2</t>
   </si>
   <si>
-    <t>C5166265</t>
+    <t>C591614</t>
   </si>
   <si>
     <t>7698</t>
@@ -788,7 +788,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1830194E-C82A-496A-BB57-D5FBA39C120E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E186953-BCA3-44B5-92EF-298DA4CF8E43}">
   <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>